<commit_message>
adapt carbon intensity assumptions
</commit_message>
<xml_diff>
--- a/input_data/Parametrization/process_parametrization.xlsx
+++ b/input_data/Parametrization/process_parametrization.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15940" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="process_techs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reference_data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="process_techs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="reference_data" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1112,7 +1112,7 @@
       <c r="D9" s="28" t="n">
         <v>25</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E9" s="22" t="n">
         <v>20</v>
       </c>
       <c r="F9" s="28" t="n">
@@ -1152,8 +1152,8 @@
       <c r="D10" s="28" t="n">
         <v>4.99</v>
       </c>
-      <c r="E10" s="28" t="n">
-        <v>20</v>
+      <c r="E10" s="22" t="n">
+        <v>59.34</v>
       </c>
       <c r="F10" s="28" t="n">
         <v>0</v>
@@ -1186,17 +1186,17 @@
           <t>ton/tonproduct</t>
         </is>
       </c>
-      <c r="C11" s="28" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D11" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="28" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F11" s="28" t="n">
-        <v>0.2</v>
+      <c r="C11" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>0</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>0.54</v>
@@ -1312,8 +1312,8 @@
       <c r="D14" s="28" t="n">
         <v>950445.42</v>
       </c>
-      <c r="E14" s="28" t="n">
-        <v>0</v>
+      <c r="E14" s="22" t="n">
+        <v>166351.72</v>
       </c>
       <c r="F14" s="28" t="n">
         <v>155954.74</v>
@@ -1394,8 +1394,8 @@
       <c r="D16" s="29" t="n">
         <v>19995771.73</v>
       </c>
-      <c r="E16" s="29" t="n">
-        <v>1363718918.918919</v>
+      <c r="E16" s="26" t="n">
+        <v>2183366.39</v>
       </c>
       <c r="F16" s="29" t="n">
         <v>3119094.84</v>

</xml_diff>

<commit_message>
fixed diffusion rate bug : now for all prod processes used inf as diffusion rate
</commit_message>
<xml_diff>
--- a/input_data/Parametrization/process_parametrization.xlsx
+++ b/input_data/Parametrization/process_parametrization.xlsx
@@ -1320,17 +1320,25 @@
           <t>1</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="E15" s="13" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="F15" s="13" t="n">
-        <v>0.13</v>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
@@ -1347,7 +1355,7 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>similar to techs existing in Crystal-Ball</t>
+          <t>baseline production tech — no diffusion bottleneck (consistent with cement_kiln, haber_bosch, olefin_from_naphtha in Crystal Ball)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
implementing feedback from jacob, jan und evren, trying to fix emission bug -> v7.2
</commit_message>
<xml_diff>
--- a/input_data/Parametrization/process_parametrization.xlsx
+++ b/input_data/Parametrization/process_parametrization.xlsx
@@ -1167,7 +1167,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="20" t="n">
-        <v>0</v>
+        <v>0.064234</v>
       </c>
       <c r="F11" s="20" t="n">
         <v>0</v>
@@ -1180,12 +1180,12 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>JRC-EU-TIMES, IPCC2006</t>
+          <t>JRC-EU-TIMES, IPCC2006, JRC BAT (ceramics)</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paper: only direct emissions from Kraft process (Calcination), which we neglect. Similar assumption to JRC-EU-TIMES model. Food: also no direct CO2 emissions (except for emissions from burning fuel and heating techs which is accounted in carriers/ heating techs). Glass: estimation of an average value of different glass types (approx. 0.2t/t), based on the assumption that there is a 50% recycling share in the EU: 0.1t/t. Ceramics: as often no carbonate (which decomposes to CO2 as in clinker production) is present in ceramic feedstocks, we assume it to be negligeble, i.e. 0t/t (based on IPCC2006) </t>
+          <t>Paper: only direct emissions from Kraft process (Calcination), which we neglect. Similar assumption to JRC-EU-TIMES model. Food: also no direct CO2 emissions (except for emissions from burning fuel and heating techs which is accounted in carriers/ heating techs). Glass: estimation of an average value of different glass types (approx. 0.2t/t), based on the assumption that there is a 50% recycling share in the EU: 0.1t/t. Ceramics: back-calculated from JRC BAT (process emissions = 15% of total ceramic emissions, remaining 85% = combustion emissions already captured by the carriers ceramic_production consumes). Combustion emissions/t = ceramic total thermal energy (8.04 GJ/t, sum of the hard_coal/natural_gas/biomass/heat_industry_0_100/heat_industry_100_200 conversion_factor rows) x weighted-average carbon intensity of the sector own hard_coal/natural_gas/biomass fuel mix, applied uniformly across all thermal energy as a representative heating tech mix (biomass treated as biogenic/zero, consistent with paper); weighted EF = 0.0453 tCO2/GJ, combustion = 0.364 tCO2/t. Process = combustion x (0.15/0.85) = 0.0642 tCO2/t. See ASSUMPTIONS.md (Ceramic).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ceramic capex assumption (based on jacobs source)
</commit_message>
<xml_diff>
--- a/input_data/Parametrization/process_parametrization.xlsx
+++ b/input_data/Parametrization/process_parametrization.xlsx
@@ -1086,8 +1086,8 @@
       <c r="D9" s="23" t="n">
         <v>25</v>
       </c>
-      <c r="E9" s="20" t="n">
-        <v>28</v>
+      <c r="E9" s="23" t="n">
+        <v>25</v>
       </c>
       <c r="F9" s="20" t="n">
         <v>20</v>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ceramics: assume similar lifespan as glass. Food: similar lifespan as steel/cement kiln. </t>
+          <t xml:space="preserve">Ceramics: 25 yr, cement-plant economic life from Gardarsdottir et al. 2019 (Energies 12, 542), reference cement plant (proxy - see assumptions.md). Food: similar lifespan as steel/cement kiln. </t>
         </is>
       </c>
     </row>
@@ -1126,8 +1126,8 @@
       <c r="D10" s="23" t="n">
         <v>4.99</v>
       </c>
-      <c r="E10" s="20" t="n">
-        <v>59.34</v>
+      <c r="E10" s="23" t="n">
+        <v>7.27</v>
       </c>
       <c r="F10" s="23" t="n">
         <v>0</v>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>Ceramics: assume similar values as glass (both use kiln)</t>
+          <t>Ceramics: 7.27 EUR/t, non-fuel variable cost (raw meal + NOx reagent + misc O&amp;M) from Gardarsdottir et al. 2019 (Energies 12, 542), reference cement plant (proxy - see assumptions.md).</t>
         </is>
       </c>
     </row>
@@ -1286,8 +1286,8 @@
       <c r="D14" s="23" t="n">
         <v>950445.42</v>
       </c>
-      <c r="E14" s="20" t="n">
-        <v>166351.72</v>
+      <c r="E14" s="23" t="n">
+        <v>156958.98</v>
       </c>
       <c r="F14" s="23" t="n">
         <v>155954.74</v>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Ceramics: assume similar values as glass (both use kiln)</t>
+          <t>Ceramics: 156,958.98 EUR/(t/h)/yr, fixed OPEX (maintenance+insurance+labor) from Gardarsdottir et al. 2019 (Energies 12, 542), reference cement plant (proxy - see assumptions.md).</t>
         </is>
       </c>
     </row>
@@ -1376,8 +1376,8 @@
       <c r="D16" s="24" t="n">
         <v>6132000</v>
       </c>
-      <c r="E16" s="22" t="n">
-        <v>2183366.39</v>
+      <c r="E16" s="24" t="n">
+        <v>1820124.59</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>3119094.84</v>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>Ceramics: assume similar values as glass (both use kiln)</t>
+          <t>Ceramics: 1,820,124.59 EUR/(t/h), CAPEX (TPC/capacity) from Gardarsdottir et al. 2019 (Energies 12, 542), reference cement plant (proxy - see assumptions.md).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adding oil as fuel input for ceramic process
</commit_message>
<xml_diff>
--- a/input_data/Parametrization/process_parametrization.xlsx
+++ b/input_data/Parametrization/process_parametrization.xlsx
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.6640625" customWidth="1" style="9" min="1" max="1"/>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>hard_coal; natural_gas; biomass; heat_industry_0_100; heat_industry_100_200; electricity</t>
+          <t>hard_coal; natural_gas; oil; biomass; heat_industry_0_100; heat_industry_100_150; heat_industry_150_200; electricity</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="D21" s="16" t="n"/>
       <c r="E21" s="16" t="n">
-        <v>0.00023638314</v>
+        <v>0.000198343232</v>
       </c>
       <c r="F21" s="16" t="n"/>
       <c r="G21" s="14" t="n"/>
@@ -1617,7 +1617,7 @@
         <v>2.2972692e-05</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>0.001002378478</v>
+        <v>0.000841070931</v>
       </c>
       <c r="F22" s="17" t="n">
         <v>4.3228709e-05</v>
@@ -1651,7 +1651,7 @@
         <v>3.3058651e-05</v>
       </c>
       <c r="E23" s="17" t="n">
-        <v>0.000496568706</v>
+        <v>0.000416658491</v>
       </c>
       <c r="F23" s="17" t="n"/>
       <c r="G23" s="17" t="n"/>
@@ -1668,41 +1668,34 @@
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>conversion_factor:heat_industry_0_100</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>GW/(tonproduct/hour)</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="n">
-        <v>2.8838889e-05</v>
-      </c>
-      <c r="D24" s="10" t="n">
-        <v>4.0022388e-05</v>
-      </c>
-      <c r="E24" s="10" t="n">
-        <v>0.000264858653</v>
-      </c>
-      <c r="F24" s="10" t="n">
-        <v>0.000292793413</v>
-      </c>
-      <c r="G24" s="10" t="n"/>
-      <c r="H24" s="10" t="n"/>
-      <c r="I24" s="7" t="inlineStr">
-        <is>
-          <t>Rehfeldt2017, AIDRES2023</t>
-        </is>
-      </c>
-      <c r="J24" s="10" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>conversion_factor:oil</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>GW/GW</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.00027925767</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Crystal Ball</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>X_production conversion_factor for oil input, written by compute_params.py</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>conversion_factor:heat_industry_100_200</t>
+          <t>conversion_factor:heat_industry_0_100</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1711,16 +1704,16 @@
         </is>
       </c>
       <c r="C25" s="10" t="n">
-        <v>0.000282621111</v>
+        <v>2.8838889e-05</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>0.001331621263</v>
+        <v>4.0022388e-05</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>0.000232147929</v>
+        <v>0.000264858653</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>0.000200917212</v>
+        <v>0.000292793413</v>
       </c>
       <c r="G25" s="10" t="n"/>
       <c r="H25" s="10" t="n"/>
@@ -1730,6 +1723,38 @@
         </is>
       </c>
       <c r="J25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>conversion_factor:heat_industry_100_200</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>GW/(tonproduct/hour)</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>0.000282621111</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>0.001331621263</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>0.000232147929</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>0.000200917212</v>
+      </c>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>Rehfeldt2017, AIDRES2023</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
first version of glass/ ceramic fuel switch
</commit_message>
<xml_diff>
--- a/input_data/Parametrization/process_parametrization.xlsx
+++ b/input_data/Parametrization/process_parametrization.xlsx
@@ -1610,15 +1610,11 @@
           <t>GW/GW</t>
         </is>
       </c>
-      <c r="C22" s="17" t="n">
-        <v>0.000932843807</v>
-      </c>
+      <c r="C22" s="17" t="n"/>
       <c r="D22" s="17" t="n">
         <v>2.2972692e-05</v>
       </c>
-      <c r="E22" s="17" t="n">
-        <v>0.000841070931</v>
-      </c>
+      <c r="E22" s="17" t="n"/>
       <c r="F22" s="17" t="n">
         <v>4.3228709e-05</v>
       </c>
@@ -1631,7 +1627,7 @@
       </c>
       <c r="J22" s="10" t="inlineStr">
         <is>
-          <t>X_production conversion_factor for natural_gas input, written by compute_params.py</t>
+          <t>No longer used as an override for glass/ceramic_production: natural_gas is now split into fuel_to_kiln (switchable) + a reduced natural_gas remainder (ceramic only), both computed dynamically by _kiln_fuel_shares() in process_parametrization.py. See ASSUMPTIONS.md, "Ceramic and glass kiln fuel switching".</t>
         </is>
       </c>
     </row>

</xml_diff>